<commit_message>
Sprint 2: Kill-Gate, Content-Klassen, Meta-Descriptions, Privacy-Hinweise
- Kill-Gate-Checkliste als Prozess-Dokument + HTML-Kommentare in Tool-Seiten
- Content-Klassen-Doku (Tool/Hub/Info/Guide/Checkliste/Legal) mit CTA-Regeln
- Privacy-Hinweise auf baby.html, einschulung.html, schatzsuche.html
- Meta-Descriptions für datenschutz, impressum, einladung, einladung/erstellen
- Richtwert-Labels in kindergeburtstag.html Planer
- Backlog Sprint 1+2 als Erledigt markiert
- validate.js: 0 Fehler, nur Warnungen

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/_dev/docs/backlog-skill-audit.xlsx
+++ b/_dev/docs/backlog-skill-audit.xlsx
@@ -587,7 +587,7 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Offen</t>
+          <t>Erledigt</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
@@ -627,7 +627,7 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>Offen</t>
+          <t>Erledigt</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -667,7 +667,7 @@
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Offen</t>
+          <t>Erledigt</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
@@ -707,7 +707,7 @@
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>Offen</t>
+          <t>Erledigt</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
@@ -747,7 +747,7 @@
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>Offen</t>
+          <t>Erledigt</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
@@ -787,7 +787,7 @@
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>Offen</t>
+          <t>Erledigt</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
@@ -827,7 +827,7 @@
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>Offen</t>
+          <t>Erledigt</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
@@ -867,7 +867,7 @@
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>Offen</t>
+          <t>Erledigt</t>
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Backlog: Sprint 3 Tasks als Erledigt markiert
Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/_dev/docs/backlog-skill-audit.xlsx
+++ b/_dev/docs/backlog-skill-audit.xlsx
@@ -907,7 +907,7 @@
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>Offen</t>
+          <t>Erledigt</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr">
@@ -947,7 +947,7 @@
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>Offen</t>
+          <t>Erledigt</t>
         </is>
       </c>
       <c r="H11" s="2" t="inlineStr">
@@ -1027,7 +1027,7 @@
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>Offen</t>
+          <t>Erledigt</t>
         </is>
       </c>
       <c r="H13" s="2" t="inlineStr">
@@ -1147,7 +1147,7 @@
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>Offen</t>
+          <t>Erledigt</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Sitemap-Automatisierung: noindex-Filter + validate.js Gate-3-Fix
- generate-sitemap.js: noindex-Seiten (datenschutz, impressum) werden ausgeschlossen
- validate.js Gate 3: überspringt noindex-Seiten beim Sitemap-Check
- Sitemap neu generiert (147 URLs, noindex-Seiten raus)
- Backlog Task 14 als Erledigt markiert

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/_dev/docs/backlog-skill-audit.xlsx
+++ b/_dev/docs/backlog-skill-audit.xlsx
@@ -1052,7 +1052,7 @@
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>Machbarkeitsanalyse: Wie sähe ein JSON + build.js-System für machsleicht aus? Welche Seiten würden profitieren? Aufwand vs. Nutzen bei aktuellem Seitenumfang (50 Seiten).</t>
+          <t>Gestrichen</t>
         </is>
       </c>
       <c r="E14" s="4" t="inlineStr">
@@ -1107,7 +1107,7 @@
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>Offen</t>
+          <t>Erledigt</t>
         </is>
       </c>
       <c r="H15" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Changelog-Kommentare eingeführt + Backlog komplett abgeschlossen
- HTML-Changelog-Kommentare bei allen geänderten Seiten ergänzt
  (404, transparenz, datenschutz, homepage, kindergeburtstag, schatzsuche)
- Backlog Task 11 → Erledigt, Task 13 → Gestrichen
- Alle 15 Backlog-Tasks nun abgeschlossen (Sprint 1-4 komplett)

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/_dev/docs/backlog-skill-audit.xlsx
+++ b/_dev/docs/backlog-skill-audit.xlsx
@@ -987,12 +987,12 @@
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>Offen</t>
+          <t>Erledigt</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>laufend</t>
+          <t>4</t>
         </is>
       </c>
     </row>
@@ -1067,7 +1067,7 @@
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>Offen</t>
+          <t>Gestrichen</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Backlog aktualisiert: 25 neue Items (Sprint 13-15 + Langfrist)
- Sprint 13: Worker Deploy, Token, GSC, Bugs
- Sprint 14: Rätsel nach Maß, Kreuzworträtsel, Awin, ElevenLabs
- Sprint 15: Standalone Wunschliste
- Backlog: KI-Spielleiter, Audio, Abo, Multiplayer, machsruhig, TeamPulse, CV Hero

Co-Authored-By: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/_dev/docs/backlog-skill-audit.xlsx
+++ b/_dev/docs/backlog-skill-audit.xlsx
@@ -19,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="14">
+  <fonts count="15">
     <font>
       <name val="Calibri"/>
       <charset val="1"/>
@@ -118,8 +118,12 @@
       <color rgb="FFE65100"/>
       <sz val="10"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+    </font>
   </fonts>
-  <fills count="9">
+  <fills count="10">
     <fill>
       <patternFill/>
     </fill>
@@ -168,6 +172,12 @@
         <bgColor rgb="FFFFF8E1"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E8873D"/>
+        <bgColor rgb="00E8873D"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="3">
     <border>
@@ -218,7 +228,7 @@
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="32">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -310,6 +320,7 @@
     <xf numFmtId="0" fontId="8" fillId="5" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="14" fillId="9" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -581,7 +592,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:H36"/>
+  <dimension ref="A1:H65"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="1" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="5" customWidth="1" style="15" min="1" max="1"/>
@@ -1928,6 +1939,984 @@
         <v>5</v>
       </c>
     </row>
+    <row r="37">
+      <c r="A37" t="inlineStr"/>
+      <c r="B37" t="inlineStr"/>
+      <c r="C37" t="inlineStr"/>
+      <c r="D37" t="inlineStr"/>
+      <c r="E37" t="inlineStr"/>
+      <c r="F37" t="inlineStr"/>
+      <c r="G37" t="inlineStr"/>
+      <c r="H37" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="31" t="inlineStr">
+        <is>
+          <t>SPRINT 13 — Partyseite + Revenue (08.04.2026)</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr"/>
+      <c r="C38" t="inlineStr"/>
+      <c r="D38" t="inlineStr"/>
+      <c r="E38" t="inlineStr"/>
+      <c r="F38" t="inlineStr"/>
+      <c r="G38" t="inlineStr"/>
+      <c r="H38" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" t="n">
+        <v>34</v>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>HOCH</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Cloudflare Worker deployen</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>party-worker.js deployen, KV 'PARTY' anlegen + binden, DNS party.machsleicht.de → Worker</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>Infrastruktur</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>1h</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>Offen</t>
+        </is>
+      </c>
+      <c r="H39" t="n">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="n">
+        <v>35</v>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>HOCH</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>AMAZON_TAG setzen</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>Amazon PartnerNet Tag als ENV var im Cloudflare Worker setzen (sobald Tag erhalten)</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>Revenue</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>5 min</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>Offen</t>
+        </is>
+      </c>
+      <c r="H40" t="n">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="n">
+        <v>36</v>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>HOCH</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Partyseite-Card Status fixen</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>Homepage index.js: Partyseite-Card zeigt 'live' → auf 'bald' setzen bis Worker deployed</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>Bug</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>10 min</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>Offen</t>
+        </is>
+      </c>
+      <c r="H41" t="n">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="n">
+        <v>37</v>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>HOCH</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Planer CTA prüfen</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>CTA '📱 Partyseite erstellen' linkt auf party.machsleicht.de → geht ins Leere bis deployed</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>Bug</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>10 min</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>Offen</t>
+        </is>
+      </c>
+      <c r="H42" t="n">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="n">
+        <v>38</v>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>HOCH</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Rätsel nach Maß</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>Eltern beschreiben Ort, Claude API generiert 5 personalisierte Rätsel. VK 2.99€. Lemon Squeezy Payment.</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>Revenue / Feature</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>4h</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>Offen</t>
+        </is>
+      </c>
+      <c r="H43" t="n">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="n">
+        <v>39</v>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>HOCH</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>GitHub Token rotieren</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>PAT für Bollesan91/machsleicht-deploy läuft am 25.04.2026 ab. Neuen Token generieren + in Netlify + lokal updaten.</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>Infrastruktur</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>15 min</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>Offen</t>
+        </is>
+      </c>
+      <c r="H44" t="n">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="n">
+        <v>40</v>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>HOCH</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Google Search Console einrichten</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>Domain verifizieren, Sitemap einreichen, Traffic-Quellen verstehen (83 UV/Tag, Herkunft unbekannt)</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>SEO</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>30 min</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>Offen</t>
+        </is>
+      </c>
+      <c r="H45" t="n">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="n">
+        <v>41</v>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>MITTEL</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>Awin anmelden</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>Publisher-Account für myToys, Thalia, Otto, Jako-o, tausendkind Affiliate. AWIN_PUBLISHER_ID als ENV var.</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>Revenue</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>1h</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>Offen</t>
+        </is>
+      </c>
+      <c r="H46" t="n">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="n">
+        <v>42</v>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>MITTEL</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>Kreuzworträtsel Premium</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>Freebie: eigene Fragen. Premium: KI generiert Inhalte passend zum Geburtstag. Upgrade von /kreuzwortraetsel.</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>Revenue / Feature</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>3h</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>Offen</t>
+        </is>
+      </c>
+      <c r="H47" t="n">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="n">
+        <v>43</v>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>MITTEL</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>Standalone /wunschliste</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>Eigene SEO-Seite, auch ohne Partyseite nutzbar. Keywords: 'Wunschliste Kind', 'Geschenke-Wunschliste'</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>SEO / Feature</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>4h</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>Offen</t>
+        </is>
+      </c>
+      <c r="H48" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="n">
+        <v>44</v>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>MITTEL</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>homepage.js aufräumen</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>Toter Partyseite-Code in homepage.js entfernen. Partyseite-Card doppelt in index.js.</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>Code-Qualität</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>30 min</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>Offen</t>
+        </is>
+      </c>
+      <c r="H49" t="n">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="n">
+        <v>45</v>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>MITTEL</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>ElevenLabs deutsche Stimmen testen</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>Bolle testet Stimmenqualität für KI-Spielleiter, Einladungs-Audio, Spielmoderation</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>Recherche</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>1h</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>Offen</t>
+        </is>
+      </c>
+      <c r="H50" t="n">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="n">
+        <v>46</v>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>MITTEL</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>Lemon Squeezy Integration</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>Payment für Rätsel nach Maß (2.99€). Checkout-Flow, Webhook, Freischaltung.</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>Revenue</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>3h</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>Offen</t>
+        </is>
+      </c>
+      <c r="H51" t="n">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="n">
+        <v>47</v>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>NIEDRIG</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>Plausible Analytics auswerten</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>Plausible ist eingebaut — Daten checken, Top-Pages, Referrer, Bounce Rate</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>Analytics</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>30 min</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>Offen</t>
+        </is>
+      </c>
+      <c r="H52" t="n">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="n">
+        <v>48</v>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>NIEDRIG</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>Inline-Styles durch CSS-Klassen ersetzen</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>242 Inline-Styles sukzessive durch Utility-Klassen ersetzen</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>Code-Qualität</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>4h</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>Offen</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr"/>
+    </row>
+    <row r="54">
+      <c r="A54" t="n">
+        <v>49</v>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>NIEDRIG</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>Sitemap bei Google einreichen</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>In GSC unter Sitemaps einreichen. Braucht GSC-Zugang (→ #40).</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>SEO</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>15 min</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>Offen</t>
+        </is>
+      </c>
+      <c r="H54" t="n">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr"/>
+      <c r="B55" t="inlineStr"/>
+      <c r="C55" t="inlineStr"/>
+      <c r="D55" t="inlineStr"/>
+      <c r="E55" t="inlineStr"/>
+      <c r="F55" t="inlineStr"/>
+      <c r="G55" t="inlineStr"/>
+      <c r="H55" t="inlineStr"/>
+    </row>
+    <row r="56">
+      <c r="A56" s="31" t="inlineStr">
+        <is>
+          <t>BACKLOG — Langfrist</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr"/>
+      <c r="C56" t="inlineStr"/>
+      <c r="D56" t="inlineStr"/>
+      <c r="E56" t="inlineStr"/>
+      <c r="F56" t="inlineStr"/>
+      <c r="G56" t="inlineStr"/>
+      <c r="H56" t="inlineStr"/>
+    </row>
+    <row r="57">
+      <c r="A57" t="n">
+        <v>50</v>
+      </c>
+      <c r="B57" s="31" t="inlineStr">
+        <is>
+          <t>BACKLOG</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>KI-Spielleiter-Anrufe</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>ElevenLabs Conversational AI, 9 Anrufe pro Schatzsuche, VK 4.99€</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>Premium</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>8h</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>Backlog</t>
+        </is>
+      </c>
+      <c r="H57" t="inlineStr"/>
+    </row>
+    <row r="58">
+      <c r="A58" t="n">
+        <v>51</v>
+      </c>
+      <c r="B58" s="31" t="inlineStr">
+        <is>
+          <t>BACKLOG</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>Einladungs-Audio</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>ElevenLabs TTS, personalisierte Audio-Nachricht per WhatsApp</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>Premium</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>3h</t>
+        </is>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>Backlog</t>
+        </is>
+      </c>
+      <c r="H58" t="inlineStr"/>
+    </row>
+    <row r="59">
+      <c r="A59" t="n">
+        <v>52</v>
+      </c>
+      <c r="B59" s="31" t="inlineStr">
+        <is>
+          <t>BACKLOG</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>Gute-Nacht-Geschichte</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>Claude API + ElevenLabs TTS, personalisiert, VK 2.99€</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>Premium</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>4h</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>Backlog</t>
+        </is>
+      </c>
+      <c r="H59" t="inlineStr"/>
+    </row>
+    <row r="60">
+      <c r="A60" t="n">
+        <v>53</v>
+      </c>
+      <c r="B60" s="31" t="inlineStr">
+        <is>
+          <t>BACKLOG</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>Sofort-Schatzsuche Abo</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>2.99€/Monat, spontane KI-Schatzsuchen, braucht Rätsel nach Maß als Basis</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>Revenue</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>6h</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>Backlog</t>
+        </is>
+      </c>
+      <c r="H60" t="inlineStr"/>
+    </row>
+    <row r="61">
+      <c r="A61" t="n">
+        <v>54</v>
+      </c>
+      <c r="B61" s="31" t="inlineStr">
+        <is>
+          <t>BACKLOG</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>Multiplayer-Schatzsuche</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>8-12 Jahre, Rollen-Links, Live-Leaderboard, WebSockets, VK 4.99€</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>Premium</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>40h</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>Backlog</t>
+        </is>
+      </c>
+      <c r="H61" t="inlineStr"/>
+    </row>
+    <row r="62">
+      <c r="A62" t="n">
+        <v>55</v>
+      </c>
+      <c r="B62" s="31" t="inlineStr">
+        <is>
+          <t>BACKLOG</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>machsruhig.de starten</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>End-of-Life/Funeral Planning, 28 Phasen, Domain gesichert</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>Neues Projekt</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>80h+</t>
+        </is>
+      </c>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>Backlog</t>
+        </is>
+      </c>
+      <c r="H62" t="inlineStr"/>
+    </row>
+    <row r="63">
+      <c r="A63" t="n">
+        <v>56</v>
+      </c>
+      <c r="B63" s="31" t="inlineStr">
+        <is>
+          <t>BACKLOG</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>TeamPulse KV Namespace</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>Cloudflare KV 'TP' anlegen + binden für Worker v2</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>Advergy</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>30 min</t>
+        </is>
+      </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>Backlog</t>
+        </is>
+      </c>
+      <c r="H63" t="inlineStr"/>
+    </row>
+    <row r="64">
+      <c r="A64" t="n">
+        <v>57</v>
+      </c>
+      <c r="B64" s="31" t="inlineStr">
+        <is>
+          <t>BACKLOG</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>TeamPulse Power Automate</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>Flow für DEALS+Invoice Sheet-Sync</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>Advergy</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>2h</t>
+        </is>
+      </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>Backlog</t>
+        </is>
+      </c>
+      <c r="H64" t="inlineStr"/>
+    </row>
+    <row r="65">
+      <c r="A65" t="n">
+        <v>58</v>
+      </c>
+      <c r="B65" s="31" t="inlineStr">
+        <is>
+          <t>BACKLOG</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>CV Hero / Fishing Ninja Cleanup</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>API Key entfernen, Mascots, Privacy Banner, +Projekt Button</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>Advergy</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>2h</t>
+        </is>
+      </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>Backlog</t>
+        </is>
+      </c>
+      <c r="H65" t="inlineStr"/>
+    </row>
   </sheetData>
   <autoFilter ref="A1:H1"/>
   <mergeCells count="1">

</xml_diff>

<commit_message>
Partyseite: 4 Bugfixes Gästeansicht (Tab-Titel-Leak, Script-Crashes, Regex-Escapes) + PBI #65 Email-Capture [skip netlify]
Co-Authored-By: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/_dev/docs/backlog-skill-audit.xlsx
+++ b/_dev/docs/backlog-skill-audit.xlsx
@@ -592,7 +592,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:H65"/>
+  <dimension ref="A1:H66"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="1" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="5" customWidth="1" style="15" min="1" max="1"/>
@@ -1247,7 +1247,6 @@
         </is>
       </c>
     </row>
-    <row r="17"/>
     <row r="18" ht="15" customHeight="1" s="16">
       <c r="A18" s="23" t="inlineStr">
         <is>
@@ -1940,14 +1939,14 @@
       </c>
     </row>
     <row r="37">
-      <c r="A37" t="inlineStr"/>
-      <c r="B37" t="inlineStr"/>
-      <c r="C37" t="inlineStr"/>
-      <c r="D37" t="inlineStr"/>
-      <c r="E37" t="inlineStr"/>
-      <c r="F37" t="inlineStr"/>
-      <c r="G37" t="inlineStr"/>
-      <c r="H37" t="inlineStr"/>
+      <c r="A37" s="15" t="inlineStr"/>
+      <c r="B37" s="15" t="inlineStr"/>
+      <c r="C37" s="15" t="inlineStr"/>
+      <c r="D37" s="15" t="inlineStr"/>
+      <c r="E37" s="15" t="inlineStr"/>
+      <c r="F37" s="15" t="inlineStr"/>
+      <c r="G37" s="15" t="inlineStr"/>
+      <c r="H37" s="15" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" s="31" t="inlineStr">
@@ -1955,629 +1954,629 @@
           <t>SPRINT 13 — Partyseite + Revenue (08.04.2026)</t>
         </is>
       </c>
-      <c r="B38" t="inlineStr"/>
-      <c r="C38" t="inlineStr"/>
-      <c r="D38" t="inlineStr"/>
-      <c r="E38" t="inlineStr"/>
-      <c r="F38" t="inlineStr"/>
-      <c r="G38" t="inlineStr"/>
-      <c r="H38" t="inlineStr"/>
+      <c r="B38" s="15" t="inlineStr"/>
+      <c r="C38" s="15" t="inlineStr"/>
+      <c r="D38" s="15" t="inlineStr"/>
+      <c r="E38" s="15" t="inlineStr"/>
+      <c r="F38" s="15" t="inlineStr"/>
+      <c r="G38" s="15" t="inlineStr"/>
+      <c r="H38" s="15" t="inlineStr"/>
     </row>
     <row r="39">
-      <c r="A39" t="n">
+      <c r="A39" s="15" t="n">
         <v>34</v>
       </c>
-      <c r="B39" t="inlineStr">
+      <c r="B39" s="15" t="inlineStr">
         <is>
           <t>HOCH</t>
         </is>
       </c>
-      <c r="C39" t="inlineStr">
+      <c r="C39" s="15" t="inlineStr">
         <is>
           <t>Cloudflare Worker deployen</t>
         </is>
       </c>
-      <c r="D39" t="inlineStr">
+      <c r="D39" s="15" t="inlineStr">
         <is>
           <t>party-worker.js deployen, KV 'PARTY' anlegen + binden, DNS party.machsleicht.de → Worker</t>
         </is>
       </c>
-      <c r="E39" t="inlineStr">
+      <c r="E39" s="15" t="inlineStr">
         <is>
           <t>Infrastruktur</t>
         </is>
       </c>
-      <c r="F39" t="inlineStr">
+      <c r="F39" s="15" t="inlineStr">
         <is>
           <t>1h</t>
         </is>
       </c>
-      <c r="G39" t="inlineStr">
+      <c r="G39" s="15" t="inlineStr">
         <is>
           <t>Offen</t>
         </is>
       </c>
-      <c r="H39" t="n">
+      <c r="H39" s="15" t="n">
         <v>13</v>
       </c>
     </row>
     <row r="40">
-      <c r="A40" t="n">
+      <c r="A40" s="15" t="n">
         <v>35</v>
       </c>
-      <c r="B40" t="inlineStr">
+      <c r="B40" s="15" t="inlineStr">
         <is>
           <t>HOCH</t>
         </is>
       </c>
-      <c r="C40" t="inlineStr">
+      <c r="C40" s="15" t="inlineStr">
         <is>
           <t>AMAZON_TAG setzen</t>
         </is>
       </c>
-      <c r="D40" t="inlineStr">
+      <c r="D40" s="15" t="inlineStr">
         <is>
           <t>Amazon PartnerNet Tag als ENV var im Cloudflare Worker setzen (sobald Tag erhalten)</t>
         </is>
       </c>
-      <c r="E40" t="inlineStr">
+      <c r="E40" s="15" t="inlineStr">
         <is>
           <t>Revenue</t>
         </is>
       </c>
-      <c r="F40" t="inlineStr">
+      <c r="F40" s="15" t="inlineStr">
         <is>
           <t>5 min</t>
         </is>
       </c>
-      <c r="G40" t="inlineStr">
+      <c r="G40" s="15" t="inlineStr">
         <is>
           <t>Offen</t>
         </is>
       </c>
-      <c r="H40" t="n">
+      <c r="H40" s="15" t="n">
         <v>13</v>
       </c>
     </row>
     <row r="41">
-      <c r="A41" t="n">
+      <c r="A41" s="15" t="n">
         <v>36</v>
       </c>
-      <c r="B41" t="inlineStr">
+      <c r="B41" s="15" t="inlineStr">
         <is>
           <t>HOCH</t>
         </is>
       </c>
-      <c r="C41" t="inlineStr">
+      <c r="C41" s="15" t="inlineStr">
         <is>
           <t>Partyseite-Card Status fixen</t>
         </is>
       </c>
-      <c r="D41" t="inlineStr">
+      <c r="D41" s="15" t="inlineStr">
         <is>
           <t>Homepage index.js: Partyseite-Card zeigt 'live' → auf 'bald' setzen bis Worker deployed</t>
         </is>
       </c>
-      <c r="E41" t="inlineStr">
+      <c r="E41" s="15" t="inlineStr">
         <is>
           <t>Bug</t>
         </is>
       </c>
-      <c r="F41" t="inlineStr">
+      <c r="F41" s="15" t="inlineStr">
         <is>
           <t>10 min</t>
         </is>
       </c>
-      <c r="G41" t="inlineStr">
+      <c r="G41" s="15" t="inlineStr">
         <is>
           <t>Offen</t>
         </is>
       </c>
-      <c r="H41" t="n">
+      <c r="H41" s="15" t="n">
         <v>13</v>
       </c>
     </row>
     <row r="42">
-      <c r="A42" t="n">
+      <c r="A42" s="15" t="n">
         <v>37</v>
       </c>
-      <c r="B42" t="inlineStr">
+      <c r="B42" s="15" t="inlineStr">
         <is>
           <t>HOCH</t>
         </is>
       </c>
-      <c r="C42" t="inlineStr">
+      <c r="C42" s="15" t="inlineStr">
         <is>
           <t>Planer CTA prüfen</t>
         </is>
       </c>
-      <c r="D42" t="inlineStr">
+      <c r="D42" s="15" t="inlineStr">
         <is>
           <t>CTA '📱 Partyseite erstellen' linkt auf party.machsleicht.de → geht ins Leere bis deployed</t>
         </is>
       </c>
-      <c r="E42" t="inlineStr">
+      <c r="E42" s="15" t="inlineStr">
         <is>
           <t>Bug</t>
         </is>
       </c>
-      <c r="F42" t="inlineStr">
+      <c r="F42" s="15" t="inlineStr">
         <is>
           <t>10 min</t>
         </is>
       </c>
-      <c r="G42" t="inlineStr">
+      <c r="G42" s="15" t="inlineStr">
         <is>
           <t>Offen</t>
         </is>
       </c>
-      <c r="H42" t="n">
+      <c r="H42" s="15" t="n">
         <v>13</v>
       </c>
     </row>
     <row r="43">
-      <c r="A43" t="n">
+      <c r="A43" s="15" t="n">
         <v>38</v>
       </c>
-      <c r="B43" t="inlineStr">
+      <c r="B43" s="15" t="inlineStr">
         <is>
           <t>HOCH</t>
         </is>
       </c>
-      <c r="C43" t="inlineStr">
+      <c r="C43" s="15" t="inlineStr">
         <is>
           <t>Rätsel nach Maß</t>
         </is>
       </c>
-      <c r="D43" t="inlineStr">
+      <c r="D43" s="15" t="inlineStr">
         <is>
           <t>Eltern beschreiben Ort, Claude API generiert 5 personalisierte Rätsel. VK 2.99€. Lemon Squeezy Payment.</t>
         </is>
       </c>
-      <c r="E43" t="inlineStr">
+      <c r="E43" s="15" t="inlineStr">
         <is>
           <t>Revenue / Feature</t>
         </is>
       </c>
-      <c r="F43" t="inlineStr">
+      <c r="F43" s="15" t="inlineStr">
         <is>
           <t>4h</t>
         </is>
       </c>
-      <c r="G43" t="inlineStr">
+      <c r="G43" s="15" t="inlineStr">
         <is>
           <t>Offen</t>
         </is>
       </c>
-      <c r="H43" t="n">
+      <c r="H43" s="15" t="n">
         <v>14</v>
       </c>
     </row>
     <row r="44">
-      <c r="A44" t="n">
+      <c r="A44" s="15" t="n">
         <v>39</v>
       </c>
-      <c r="B44" t="inlineStr">
+      <c r="B44" s="15" t="inlineStr">
         <is>
           <t>HOCH</t>
         </is>
       </c>
-      <c r="C44" t="inlineStr">
+      <c r="C44" s="15" t="inlineStr">
         <is>
           <t>GitHub Token rotieren</t>
         </is>
       </c>
-      <c r="D44" t="inlineStr">
+      <c r="D44" s="15" t="inlineStr">
         <is>
           <t>PAT für Bollesan91/machsleicht-deploy läuft am 25.04.2026 ab. Neuen Token generieren + in Netlify + lokal updaten.</t>
         </is>
       </c>
-      <c r="E44" t="inlineStr">
+      <c r="E44" s="15" t="inlineStr">
         <is>
           <t>Infrastruktur</t>
         </is>
       </c>
-      <c r="F44" t="inlineStr">
+      <c r="F44" s="15" t="inlineStr">
         <is>
           <t>15 min</t>
         </is>
       </c>
-      <c r="G44" t="inlineStr">
+      <c r="G44" s="15" t="inlineStr">
         <is>
           <t>Offen</t>
         </is>
       </c>
-      <c r="H44" t="n">
+      <c r="H44" s="15" t="n">
         <v>13</v>
       </c>
     </row>
     <row r="45">
-      <c r="A45" t="n">
+      <c r="A45" s="15" t="n">
         <v>40</v>
       </c>
-      <c r="B45" t="inlineStr">
+      <c r="B45" s="15" t="inlineStr">
         <is>
           <t>HOCH</t>
         </is>
       </c>
-      <c r="C45" t="inlineStr">
+      <c r="C45" s="15" t="inlineStr">
         <is>
           <t>Google Search Console einrichten</t>
         </is>
       </c>
-      <c r="D45" t="inlineStr">
+      <c r="D45" s="15" t="inlineStr">
         <is>
           <t>Domain verifizieren, Sitemap einreichen, Traffic-Quellen verstehen (83 UV/Tag, Herkunft unbekannt)</t>
         </is>
       </c>
-      <c r="E45" t="inlineStr">
+      <c r="E45" s="15" t="inlineStr">
         <is>
           <t>SEO</t>
         </is>
       </c>
-      <c r="F45" t="inlineStr">
+      <c r="F45" s="15" t="inlineStr">
         <is>
           <t>30 min</t>
         </is>
       </c>
-      <c r="G45" t="inlineStr">
+      <c r="G45" s="15" t="inlineStr">
         <is>
           <t>Offen</t>
         </is>
       </c>
-      <c r="H45" t="n">
+      <c r="H45" s="15" t="n">
         <v>13</v>
       </c>
     </row>
     <row r="46">
-      <c r="A46" t="n">
+      <c r="A46" s="15" t="n">
         <v>41</v>
       </c>
-      <c r="B46" t="inlineStr">
+      <c r="B46" s="15" t="inlineStr">
         <is>
           <t>MITTEL</t>
         </is>
       </c>
-      <c r="C46" t="inlineStr">
+      <c r="C46" s="15" t="inlineStr">
         <is>
           <t>Awin anmelden</t>
         </is>
       </c>
-      <c r="D46" t="inlineStr">
+      <c r="D46" s="15" t="inlineStr">
         <is>
           <t>Publisher-Account für myToys, Thalia, Otto, Jako-o, tausendkind Affiliate. AWIN_PUBLISHER_ID als ENV var.</t>
         </is>
       </c>
-      <c r="E46" t="inlineStr">
+      <c r="E46" s="15" t="inlineStr">
         <is>
           <t>Revenue</t>
         </is>
       </c>
-      <c r="F46" t="inlineStr">
+      <c r="F46" s="15" t="inlineStr">
         <is>
           <t>1h</t>
         </is>
       </c>
-      <c r="G46" t="inlineStr">
+      <c r="G46" s="15" t="inlineStr">
         <is>
           <t>Offen</t>
         </is>
       </c>
-      <c r="H46" t="n">
+      <c r="H46" s="15" t="n">
         <v>14</v>
       </c>
     </row>
     <row r="47">
-      <c r="A47" t="n">
+      <c r="A47" s="15" t="n">
         <v>42</v>
       </c>
-      <c r="B47" t="inlineStr">
+      <c r="B47" s="15" t="inlineStr">
         <is>
           <t>MITTEL</t>
         </is>
       </c>
-      <c r="C47" t="inlineStr">
+      <c r="C47" s="15" t="inlineStr">
         <is>
           <t>Kreuzworträtsel Premium</t>
         </is>
       </c>
-      <c r="D47" t="inlineStr">
+      <c r="D47" s="15" t="inlineStr">
         <is>
           <t>Freebie: eigene Fragen. Premium: KI generiert Inhalte passend zum Geburtstag. Upgrade von /kreuzwortraetsel.</t>
         </is>
       </c>
-      <c r="E47" t="inlineStr">
+      <c r="E47" s="15" t="inlineStr">
         <is>
           <t>Revenue / Feature</t>
         </is>
       </c>
-      <c r="F47" t="inlineStr">
+      <c r="F47" s="15" t="inlineStr">
         <is>
           <t>3h</t>
         </is>
       </c>
-      <c r="G47" t="inlineStr">
+      <c r="G47" s="15" t="inlineStr">
         <is>
           <t>Offen</t>
         </is>
       </c>
-      <c r="H47" t="n">
+      <c r="H47" s="15" t="n">
         <v>14</v>
       </c>
     </row>
     <row r="48">
-      <c r="A48" t="n">
+      <c r="A48" s="15" t="n">
         <v>43</v>
       </c>
-      <c r="B48" t="inlineStr">
+      <c r="B48" s="15" t="inlineStr">
         <is>
           <t>MITTEL</t>
         </is>
       </c>
-      <c r="C48" t="inlineStr">
+      <c r="C48" s="15" t="inlineStr">
         <is>
           <t>Standalone /wunschliste</t>
         </is>
       </c>
-      <c r="D48" t="inlineStr">
+      <c r="D48" s="15" t="inlineStr">
         <is>
           <t>Eigene SEO-Seite, auch ohne Partyseite nutzbar. Keywords: 'Wunschliste Kind', 'Geschenke-Wunschliste'</t>
         </is>
       </c>
-      <c r="E48" t="inlineStr">
+      <c r="E48" s="15" t="inlineStr">
         <is>
           <t>SEO / Feature</t>
         </is>
       </c>
-      <c r="F48" t="inlineStr">
+      <c r="F48" s="15" t="inlineStr">
         <is>
           <t>4h</t>
         </is>
       </c>
-      <c r="G48" t="inlineStr">
+      <c r="G48" s="15" t="inlineStr">
         <is>
           <t>Offen</t>
         </is>
       </c>
-      <c r="H48" t="n">
+      <c r="H48" s="15" t="n">
         <v>15</v>
       </c>
     </row>
     <row r="49">
-      <c r="A49" t="n">
+      <c r="A49" s="15" t="n">
         <v>44</v>
       </c>
-      <c r="B49" t="inlineStr">
+      <c r="B49" s="15" t="inlineStr">
         <is>
           <t>MITTEL</t>
         </is>
       </c>
-      <c r="C49" t="inlineStr">
+      <c r="C49" s="15" t="inlineStr">
         <is>
           <t>homepage.js aufräumen</t>
         </is>
       </c>
-      <c r="D49" t="inlineStr">
+      <c r="D49" s="15" t="inlineStr">
         <is>
           <t>Toter Partyseite-Code in homepage.js entfernen. Partyseite-Card doppelt in index.js.</t>
         </is>
       </c>
-      <c r="E49" t="inlineStr">
+      <c r="E49" s="15" t="inlineStr">
         <is>
           <t>Code-Qualität</t>
         </is>
       </c>
-      <c r="F49" t="inlineStr">
+      <c r="F49" s="15" t="inlineStr">
         <is>
           <t>30 min</t>
         </is>
       </c>
-      <c r="G49" t="inlineStr">
+      <c r="G49" s="15" t="inlineStr">
         <is>
           <t>Offen</t>
         </is>
       </c>
-      <c r="H49" t="n">
+      <c r="H49" s="15" t="n">
         <v>13</v>
       </c>
     </row>
     <row r="50">
-      <c r="A50" t="n">
+      <c r="A50" s="15" t="n">
         <v>45</v>
       </c>
-      <c r="B50" t="inlineStr">
+      <c r="B50" s="15" t="inlineStr">
         <is>
           <t>MITTEL</t>
         </is>
       </c>
-      <c r="C50" t="inlineStr">
+      <c r="C50" s="15" t="inlineStr">
         <is>
           <t>ElevenLabs deutsche Stimmen testen</t>
         </is>
       </c>
-      <c r="D50" t="inlineStr">
+      <c r="D50" s="15" t="inlineStr">
         <is>
           <t>Bolle testet Stimmenqualität für KI-Spielleiter, Einladungs-Audio, Spielmoderation</t>
         </is>
       </c>
-      <c r="E50" t="inlineStr">
+      <c r="E50" s="15" t="inlineStr">
         <is>
           <t>Recherche</t>
         </is>
       </c>
-      <c r="F50" t="inlineStr">
+      <c r="F50" s="15" t="inlineStr">
         <is>
           <t>1h</t>
         </is>
       </c>
-      <c r="G50" t="inlineStr">
+      <c r="G50" s="15" t="inlineStr">
         <is>
           <t>Offen</t>
         </is>
       </c>
-      <c r="H50" t="n">
+      <c r="H50" s="15" t="n">
         <v>14</v>
       </c>
     </row>
     <row r="51">
-      <c r="A51" t="n">
+      <c r="A51" s="15" t="n">
         <v>46</v>
       </c>
-      <c r="B51" t="inlineStr">
+      <c r="B51" s="15" t="inlineStr">
         <is>
           <t>MITTEL</t>
         </is>
       </c>
-      <c r="C51" t="inlineStr">
+      <c r="C51" s="15" t="inlineStr">
         <is>
           <t>Lemon Squeezy Integration</t>
         </is>
       </c>
-      <c r="D51" t="inlineStr">
+      <c r="D51" s="15" t="inlineStr">
         <is>
           <t>Payment für Rätsel nach Maß (2.99€). Checkout-Flow, Webhook, Freischaltung.</t>
         </is>
       </c>
-      <c r="E51" t="inlineStr">
+      <c r="E51" s="15" t="inlineStr">
         <is>
           <t>Revenue</t>
         </is>
       </c>
-      <c r="F51" t="inlineStr">
+      <c r="F51" s="15" t="inlineStr">
         <is>
           <t>3h</t>
         </is>
       </c>
-      <c r="G51" t="inlineStr">
+      <c r="G51" s="15" t="inlineStr">
         <is>
           <t>Offen</t>
         </is>
       </c>
-      <c r="H51" t="n">
+      <c r="H51" s="15" t="n">
         <v>14</v>
       </c>
     </row>
     <row r="52">
-      <c r="A52" t="n">
+      <c r="A52" s="15" t="n">
         <v>47</v>
       </c>
-      <c r="B52" t="inlineStr">
+      <c r="B52" s="15" t="inlineStr">
         <is>
           <t>NIEDRIG</t>
         </is>
       </c>
-      <c r="C52" t="inlineStr">
+      <c r="C52" s="15" t="inlineStr">
         <is>
           <t>Plausible Analytics auswerten</t>
         </is>
       </c>
-      <c r="D52" t="inlineStr">
+      <c r="D52" s="15" t="inlineStr">
         <is>
           <t>Plausible ist eingebaut — Daten checken, Top-Pages, Referrer, Bounce Rate</t>
         </is>
       </c>
-      <c r="E52" t="inlineStr">
+      <c r="E52" s="15" t="inlineStr">
         <is>
           <t>Analytics</t>
         </is>
       </c>
-      <c r="F52" t="inlineStr">
+      <c r="F52" s="15" t="inlineStr">
         <is>
           <t>30 min</t>
         </is>
       </c>
-      <c r="G52" t="inlineStr">
+      <c r="G52" s="15" t="inlineStr">
         <is>
           <t>Offen</t>
         </is>
       </c>
-      <c r="H52" t="n">
+      <c r="H52" s="15" t="n">
         <v>13</v>
       </c>
     </row>
     <row r="53">
-      <c r="A53" t="n">
+      <c r="A53" s="15" t="n">
         <v>48</v>
       </c>
-      <c r="B53" t="inlineStr">
+      <c r="B53" s="15" t="inlineStr">
         <is>
           <t>NIEDRIG</t>
         </is>
       </c>
-      <c r="C53" t="inlineStr">
+      <c r="C53" s="15" t="inlineStr">
         <is>
           <t>Inline-Styles durch CSS-Klassen ersetzen</t>
         </is>
       </c>
-      <c r="D53" t="inlineStr">
+      <c r="D53" s="15" t="inlineStr">
         <is>
           <t>242 Inline-Styles sukzessive durch Utility-Klassen ersetzen</t>
         </is>
       </c>
-      <c r="E53" t="inlineStr">
+      <c r="E53" s="15" t="inlineStr">
         <is>
           <t>Code-Qualität</t>
         </is>
       </c>
-      <c r="F53" t="inlineStr">
+      <c r="F53" s="15" t="inlineStr">
         <is>
           <t>4h</t>
         </is>
       </c>
-      <c r="G53" t="inlineStr">
+      <c r="G53" s="15" t="inlineStr">
         <is>
           <t>Offen</t>
         </is>
       </c>
-      <c r="H53" t="inlineStr"/>
+      <c r="H53" s="15" t="inlineStr"/>
     </row>
     <row r="54">
-      <c r="A54" t="n">
+      <c r="A54" s="15" t="n">
         <v>49</v>
       </c>
-      <c r="B54" t="inlineStr">
+      <c r="B54" s="15" t="inlineStr">
         <is>
           <t>NIEDRIG</t>
         </is>
       </c>
-      <c r="C54" t="inlineStr">
+      <c r="C54" s="15" t="inlineStr">
         <is>
           <t>Sitemap bei Google einreichen</t>
         </is>
       </c>
-      <c r="D54" t="inlineStr">
+      <c r="D54" s="15" t="inlineStr">
         <is>
           <t>In GSC unter Sitemaps einreichen. Braucht GSC-Zugang (→ #40).</t>
         </is>
       </c>
-      <c r="E54" t="inlineStr">
+      <c r="E54" s="15" t="inlineStr">
         <is>
           <t>SEO</t>
         </is>
       </c>
-      <c r="F54" t="inlineStr">
+      <c r="F54" s="15" t="inlineStr">
         <is>
           <t>15 min</t>
         </is>
       </c>
-      <c r="G54" t="inlineStr">
+      <c r="G54" s="15" t="inlineStr">
         <is>
           <t>Offen</t>
         </is>
       </c>
-      <c r="H54" t="n">
+      <c r="H54" s="15" t="n">
         <v>13</v>
       </c>
     </row>
     <row r="55">
-      <c r="A55" t="inlineStr"/>
-      <c r="B55" t="inlineStr"/>
-      <c r="C55" t="inlineStr"/>
-      <c r="D55" t="inlineStr"/>
-      <c r="E55" t="inlineStr"/>
-      <c r="F55" t="inlineStr"/>
-      <c r="G55" t="inlineStr"/>
-      <c r="H55" t="inlineStr"/>
+      <c r="A55" s="15" t="inlineStr"/>
+      <c r="B55" s="15" t="inlineStr"/>
+      <c r="C55" s="15" t="inlineStr"/>
+      <c r="D55" s="15" t="inlineStr"/>
+      <c r="E55" s="15" t="inlineStr"/>
+      <c r="F55" s="15" t="inlineStr"/>
+      <c r="G55" s="15" t="inlineStr"/>
+      <c r="H55" s="15" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" s="31" t="inlineStr">
@@ -2585,16 +2584,16 @@
           <t>BACKLOG — Langfrist</t>
         </is>
       </c>
-      <c r="B56" t="inlineStr"/>
-      <c r="C56" t="inlineStr"/>
-      <c r="D56" t="inlineStr"/>
-      <c r="E56" t="inlineStr"/>
-      <c r="F56" t="inlineStr"/>
-      <c r="G56" t="inlineStr"/>
-      <c r="H56" t="inlineStr"/>
+      <c r="B56" s="15" t="inlineStr"/>
+      <c r="C56" s="15" t="inlineStr"/>
+      <c r="D56" s="15" t="inlineStr"/>
+      <c r="E56" s="15" t="inlineStr"/>
+      <c r="F56" s="15" t="inlineStr"/>
+      <c r="G56" s="15" t="inlineStr"/>
+      <c r="H56" s="15" t="inlineStr"/>
     </row>
     <row r="57">
-      <c r="A57" t="n">
+      <c r="A57" s="15" t="n">
         <v>50</v>
       </c>
       <c r="B57" s="31" t="inlineStr">
@@ -2602,35 +2601,35 @@
           <t>BACKLOG</t>
         </is>
       </c>
-      <c r="C57" t="inlineStr">
+      <c r="C57" s="15" t="inlineStr">
         <is>
           <t>KI-Spielleiter-Anrufe</t>
         </is>
       </c>
-      <c r="D57" t="inlineStr">
+      <c r="D57" s="15" t="inlineStr">
         <is>
           <t>ElevenLabs Conversational AI, 9 Anrufe pro Schatzsuche, VK 4.99€</t>
         </is>
       </c>
-      <c r="E57" t="inlineStr">
+      <c r="E57" s="15" t="inlineStr">
         <is>
           <t>Premium</t>
         </is>
       </c>
-      <c r="F57" t="inlineStr">
+      <c r="F57" s="15" t="inlineStr">
         <is>
           <t>8h</t>
         </is>
       </c>
-      <c r="G57" t="inlineStr">
+      <c r="G57" s="15" t="inlineStr">
         <is>
           <t>Backlog</t>
         </is>
       </c>
-      <c r="H57" t="inlineStr"/>
+      <c r="H57" s="15" t="inlineStr"/>
     </row>
     <row r="58">
-      <c r="A58" t="n">
+      <c r="A58" s="15" t="n">
         <v>51</v>
       </c>
       <c r="B58" s="31" t="inlineStr">
@@ -2638,35 +2637,35 @@
           <t>BACKLOG</t>
         </is>
       </c>
-      <c r="C58" t="inlineStr">
+      <c r="C58" s="15" t="inlineStr">
         <is>
           <t>Einladungs-Audio</t>
         </is>
       </c>
-      <c r="D58" t="inlineStr">
+      <c r="D58" s="15" t="inlineStr">
         <is>
           <t>ElevenLabs TTS, personalisierte Audio-Nachricht per WhatsApp</t>
         </is>
       </c>
-      <c r="E58" t="inlineStr">
+      <c r="E58" s="15" t="inlineStr">
         <is>
           <t>Premium</t>
         </is>
       </c>
-      <c r="F58" t="inlineStr">
+      <c r="F58" s="15" t="inlineStr">
         <is>
           <t>3h</t>
         </is>
       </c>
-      <c r="G58" t="inlineStr">
+      <c r="G58" s="15" t="inlineStr">
         <is>
           <t>Backlog</t>
         </is>
       </c>
-      <c r="H58" t="inlineStr"/>
+      <c r="H58" s="15" t="inlineStr"/>
     </row>
     <row r="59">
-      <c r="A59" t="n">
+      <c r="A59" s="15" t="n">
         <v>52</v>
       </c>
       <c r="B59" s="31" t="inlineStr">
@@ -2674,35 +2673,35 @@
           <t>BACKLOG</t>
         </is>
       </c>
-      <c r="C59" t="inlineStr">
+      <c r="C59" s="15" t="inlineStr">
         <is>
           <t>Gute-Nacht-Geschichte</t>
         </is>
       </c>
-      <c r="D59" t="inlineStr">
+      <c r="D59" s="15" t="inlineStr">
         <is>
           <t>Claude API + ElevenLabs TTS, personalisiert, VK 2.99€</t>
         </is>
       </c>
-      <c r="E59" t="inlineStr">
+      <c r="E59" s="15" t="inlineStr">
         <is>
           <t>Premium</t>
         </is>
       </c>
-      <c r="F59" t="inlineStr">
+      <c r="F59" s="15" t="inlineStr">
         <is>
           <t>4h</t>
         </is>
       </c>
-      <c r="G59" t="inlineStr">
+      <c r="G59" s="15" t="inlineStr">
         <is>
           <t>Backlog</t>
         </is>
       </c>
-      <c r="H59" t="inlineStr"/>
+      <c r="H59" s="15" t="inlineStr"/>
     </row>
     <row r="60">
-      <c r="A60" t="n">
+      <c r="A60" s="15" t="n">
         <v>53</v>
       </c>
       <c r="B60" s="31" t="inlineStr">
@@ -2710,35 +2709,35 @@
           <t>BACKLOG</t>
         </is>
       </c>
-      <c r="C60" t="inlineStr">
+      <c r="C60" s="15" t="inlineStr">
         <is>
           <t>Sofort-Schatzsuche Abo</t>
         </is>
       </c>
-      <c r="D60" t="inlineStr">
+      <c r="D60" s="15" t="inlineStr">
         <is>
           <t>2.99€/Monat, spontane KI-Schatzsuchen, braucht Rätsel nach Maß als Basis</t>
         </is>
       </c>
-      <c r="E60" t="inlineStr">
+      <c r="E60" s="15" t="inlineStr">
         <is>
           <t>Revenue</t>
         </is>
       </c>
-      <c r="F60" t="inlineStr">
+      <c r="F60" s="15" t="inlineStr">
         <is>
           <t>6h</t>
         </is>
       </c>
-      <c r="G60" t="inlineStr">
+      <c r="G60" s="15" t="inlineStr">
         <is>
           <t>Backlog</t>
         </is>
       </c>
-      <c r="H60" t="inlineStr"/>
+      <c r="H60" s="15" t="inlineStr"/>
     </row>
     <row r="61">
-      <c r="A61" t="n">
+      <c r="A61" s="15" t="n">
         <v>54</v>
       </c>
       <c r="B61" s="31" t="inlineStr">
@@ -2746,35 +2745,35 @@
           <t>BACKLOG</t>
         </is>
       </c>
-      <c r="C61" t="inlineStr">
+      <c r="C61" s="15" t="inlineStr">
         <is>
           <t>Multiplayer-Schatzsuche</t>
         </is>
       </c>
-      <c r="D61" t="inlineStr">
+      <c r="D61" s="15" t="inlineStr">
         <is>
           <t>8-12 Jahre, Rollen-Links, Live-Leaderboard, WebSockets, VK 4.99€</t>
         </is>
       </c>
-      <c r="E61" t="inlineStr">
+      <c r="E61" s="15" t="inlineStr">
         <is>
           <t>Premium</t>
         </is>
       </c>
-      <c r="F61" t="inlineStr">
+      <c r="F61" s="15" t="inlineStr">
         <is>
           <t>40h</t>
         </is>
       </c>
-      <c r="G61" t="inlineStr">
+      <c r="G61" s="15" t="inlineStr">
         <is>
           <t>Backlog</t>
         </is>
       </c>
-      <c r="H61" t="inlineStr"/>
+      <c r="H61" s="15" t="inlineStr"/>
     </row>
     <row r="62">
-      <c r="A62" t="n">
+      <c r="A62" s="15" t="n">
         <v>55</v>
       </c>
       <c r="B62" s="31" t="inlineStr">
@@ -2782,35 +2781,35 @@
           <t>BACKLOG</t>
         </is>
       </c>
-      <c r="C62" t="inlineStr">
+      <c r="C62" s="15" t="inlineStr">
         <is>
           <t>machsruhig.de starten</t>
         </is>
       </c>
-      <c r="D62" t="inlineStr">
+      <c r="D62" s="15" t="inlineStr">
         <is>
           <t>End-of-Life/Funeral Planning, 28 Phasen, Domain gesichert</t>
         </is>
       </c>
-      <c r="E62" t="inlineStr">
+      <c r="E62" s="15" t="inlineStr">
         <is>
           <t>Neues Projekt</t>
         </is>
       </c>
-      <c r="F62" t="inlineStr">
+      <c r="F62" s="15" t="inlineStr">
         <is>
           <t>80h+</t>
         </is>
       </c>
-      <c r="G62" t="inlineStr">
+      <c r="G62" s="15" t="inlineStr">
         <is>
           <t>Backlog</t>
         </is>
       </c>
-      <c r="H62" t="inlineStr"/>
+      <c r="H62" s="15" t="inlineStr"/>
     </row>
     <row r="63">
-      <c r="A63" t="n">
+      <c r="A63" s="15" t="n">
         <v>56</v>
       </c>
       <c r="B63" s="31" t="inlineStr">
@@ -2818,35 +2817,35 @@
           <t>BACKLOG</t>
         </is>
       </c>
-      <c r="C63" t="inlineStr">
+      <c r="C63" s="15" t="inlineStr">
         <is>
           <t>TeamPulse KV Namespace</t>
         </is>
       </c>
-      <c r="D63" t="inlineStr">
+      <c r="D63" s="15" t="inlineStr">
         <is>
           <t>Cloudflare KV 'TP' anlegen + binden für Worker v2</t>
         </is>
       </c>
-      <c r="E63" t="inlineStr">
+      <c r="E63" s="15" t="inlineStr">
         <is>
           <t>Advergy</t>
         </is>
       </c>
-      <c r="F63" t="inlineStr">
+      <c r="F63" s="15" t="inlineStr">
         <is>
           <t>30 min</t>
         </is>
       </c>
-      <c r="G63" t="inlineStr">
+      <c r="G63" s="15" t="inlineStr">
         <is>
           <t>Backlog</t>
         </is>
       </c>
-      <c r="H63" t="inlineStr"/>
+      <c r="H63" s="15" t="inlineStr"/>
     </row>
     <row r="64">
-      <c r="A64" t="n">
+      <c r="A64" s="15" t="n">
         <v>57</v>
       </c>
       <c r="B64" s="31" t="inlineStr">
@@ -2854,35 +2853,35 @@
           <t>BACKLOG</t>
         </is>
       </c>
-      <c r="C64" t="inlineStr">
+      <c r="C64" s="15" t="inlineStr">
         <is>
           <t>TeamPulse Power Automate</t>
         </is>
       </c>
-      <c r="D64" t="inlineStr">
+      <c r="D64" s="15" t="inlineStr">
         <is>
           <t>Flow für DEALS+Invoice Sheet-Sync</t>
         </is>
       </c>
-      <c r="E64" t="inlineStr">
+      <c r="E64" s="15" t="inlineStr">
         <is>
           <t>Advergy</t>
         </is>
       </c>
-      <c r="F64" t="inlineStr">
+      <c r="F64" s="15" t="inlineStr">
         <is>
           <t>2h</t>
         </is>
       </c>
-      <c r="G64" t="inlineStr">
+      <c r="G64" s="15" t="inlineStr">
         <is>
           <t>Backlog</t>
         </is>
       </c>
-      <c r="H64" t="inlineStr"/>
+      <c r="H64" s="15" t="inlineStr"/>
     </row>
     <row r="65">
-      <c r="A65" t="n">
+      <c r="A65" s="15" t="n">
         <v>58</v>
       </c>
       <c r="B65" s="31" t="inlineStr">
@@ -2890,32 +2889,84 @@
           <t>BACKLOG</t>
         </is>
       </c>
-      <c r="C65" t="inlineStr">
+      <c r="C65" s="15" t="inlineStr">
         <is>
           <t>CV Hero / Fishing Ninja Cleanup</t>
         </is>
       </c>
-      <c r="D65" t="inlineStr">
+      <c r="D65" s="15" t="inlineStr">
         <is>
           <t>API Key entfernen, Mascots, Privacy Banner, +Projekt Button</t>
         </is>
       </c>
-      <c r="E65" t="inlineStr">
+      <c r="E65" s="15" t="inlineStr">
         <is>
           <t>Advergy</t>
         </is>
       </c>
-      <c r="F65" t="inlineStr">
+      <c r="F65" s="15" t="inlineStr">
         <is>
           <t>2h</t>
         </is>
       </c>
-      <c r="G65" t="inlineStr">
+      <c r="G65" s="15" t="inlineStr">
         <is>
           <t>Backlog</t>
         </is>
       </c>
-      <c r="H65" t="inlineStr"/>
+      <c r="H65" s="15" t="inlineStr"/>
+    </row>
+    <row r="66">
+      <c r="A66" t="n">
+        <v>65</v>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>Email-Capture: 5 Touchpoints + MailerLite + DSGVO</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>5 Capture-Punkte:
+1. Creator-Partyseite: "Zusagen-Updates per Mail" (Tag: creator-party)
+2. Creator-Einladung: "Link per Mail sichern" (Tag: creator-einladung)
+3. Creator-Schatzsuche: "Karte per Mail sichern" (Tag: creator-schatzsuche)
+4. Creator-Planer: "Erinnerung vor dem Geburtstag" (Tag: creator-planer)
+5. Gast-Partyseite nach RSVP: "Auch einen Geburtstag? Wir erinnern euch" (Tag: gast-reminder)
++ Einladung Gast-CTA: Simpler Link "Eigene Einladung erstellen" (kein Email-Feld)
+Technik:
+- MailerLite Account + API-Key + Custom Domain (party@machsleicht.de)
+- DNS: SPF/DKIM/DMARC via Cloudflare
+- Double-Opt-In aktivieren
+- Datenschutzseite um MailerLite-Abschnitt ergänzen
+- Ein generischer API-Endpoint für alle Captures (Tag + Custom Fields)
+Automations (Phase 2):
+- Partyseite: "Neue Zusage"-Notification
+- Gast-Reminder: Erinnerung 6 Wochen vor Kindergeburtstag
+- Creator: Erinnerung 3 Tage vor Party mit Checkliste
+Zufriedenheits-Score: 85% ohne Automations, 100% mit.</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>Growth / Retention</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>4h</t>
+        </is>
+      </c>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>Backlog</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:H1"/>

</xml_diff>